<commit_message>
(NCIOCPL#80) Search Engine Restriction tests give a false failure.
Incidental: Change YAML content request to static content.
</commit_message>
<xml_diff>
--- a/test-data/searchenginerestrictions_data.xlsx
+++ b/test-data/searchenginerestrictions_data.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10512"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06E9D360-707F-456D-A52A-E1E61044DD03}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE70E61C-7B8E-2945-8371-D5B62D7B7EC4}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="24460" yWindow="980" windowWidth="22260" windowHeight="12640" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="getpages_with_index" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="10">
   <si>
     <t>path</t>
   </si>
@@ -51,12 +51,6 @@
   </si>
   <si>
     <t>Blog Post</t>
-  </si>
-  <si>
-    <t>/about-cancer/causes-prevention/vitamin-d-fact-sheet</t>
-  </si>
-  <si>
-    <t>/about-cancer/coping/self-image</t>
   </si>
 </sst>
 </file>
@@ -384,14 +378,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="56.85546875" customWidth="1"/>
-    <col min="2" max="2" width="25.42578125" customWidth="1"/>
-    <col min="3" max="3" width="13.85546875" customWidth="1"/>
+    <col min="1" max="1" width="56.83203125" customWidth="1"/>
+    <col min="2" max="2" width="25.5" customWidth="1"/>
+    <col min="3" max="3" width="13.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -402,7 +396,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -413,7 +407,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>6</v>
       </c>
@@ -424,7 +418,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -443,14 +437,14 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C5FD1206-3591-4D75-B37B-F40530826E59}">
-  <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:C1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="19.85546875" customWidth="1"/>
-    <col min="2" max="2" width="15.28515625" customWidth="1"/>
+    <col min="1" max="1" width="19.83203125" customWidth="1"/>
+    <col min="2" max="2" width="15.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -459,28 +453,6 @@
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>10</v>
-      </c>
-      <c r="B2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>11</v>
-      </c>
-      <c r="B3" t="s">
-        <v>4</v>
-      </c>
-      <c r="C3" t="s">
-        <v>5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>